<commit_message>
fix(ui): ensure filter popup stays closed by default by checking computed style
</commit_message>
<xml_diff>
--- a/output_030822.xlsx
+++ b/output_030822.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT146"/>
+  <dimension ref="A1:AY146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -657,6 +657,31 @@
       <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>跟价店</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>沃玛希新增</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>犀牛新增</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>AA百货新增</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>1三级类目</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>2三级类目</t>
         </is>
       </c>
     </row>
@@ -795,6 +820,11 @@
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -935,6 +965,15 @@
           <t>沃玛希</t>
         </is>
       </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1075,6 +1114,15 @@
           <t>沃玛希</t>
         </is>
       </c>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1201,12 +1249,21 @@
         <v>0</v>
       </c>
       <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="AP5" t="inlineStr"/>
       <c r="AQ5" t="inlineStr"/>
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="inlineStr"/>
       <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1266,35 +1323,35 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>35006205861</v>
+        <v>42127537259</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>http://p0.meituan.net/sgopen/793d2535f74d5b8204de55f45c519027174496.jpg.webp</t>
+          <t>http://p0.meituan.net/sgopen/9c83a6c06e31ecfbde92a873e3277ed3269643.jpg.webp</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>佑亿派 香葱王薄脆饼干超薄小饼干休闲零食香葱味 口味随机8g/袋</t>
+          <t>新款元旦新年红色毛绒星星发夹女 bb夹新年蝴蝶结刘海夹侧边发卡节日氛围感头饰发饰</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>8g*1袋</t>
+          <t>3个</t>
         </is>
       </c>
       <c r="W6" t="inlineStr"/>
       <c r="X6" t="inlineStr"/>
       <c r="Y6" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="n">
-        <v>0.9788377285003662</v>
+        <v>1</v>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>图片匹配</t>
+          <t>手动关联</t>
         </is>
       </c>
       <c r="AC6" t="n">
@@ -1333,12 +1390,25 @@
         <v>0</v>
       </c>
       <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="AP6" t="inlineStr"/>
       <c r="AQ6" t="inlineStr"/>
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="inlineStr"/>
       <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>发饰</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1471,6 +1541,11 @@
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1562,35 +1637,35 @@
         </is>
       </c>
       <c r="AC8" t="n">
-        <v>44557356462</v>
+        <v>42547326062</v>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>http://p0.meituan.net/sgopen/d7211ac1aa94d7ddf73ca5a125a99a7a152589.jpg.webp</t>
+          <t>http://p0.meituan.net/sgopen/ad27c3dbea9c23bfeefc8c38e78b27d1548433.png.webp</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>比比赞 黑松露火腿苏打饼干 咸味酥脆休闲解馋健康零食品充饥早餐约20g/袋</t>
+          <t>【10份装】比比赞 爆浆曲奇小丸子巧克力夹心网红爆款小零食 约10g*10袋</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>约20g/袋</t>
+          <t>约10g*10袋</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ8" t="inlineStr"/>
       <c r="AK8" t="n">
-        <v>0.7849698662757874</v>
+        <v>1</v>
       </c>
       <c r="AL8" t="inlineStr">
         <is>
-          <t>图片匹配</t>
+          <t>手动关联</t>
         </is>
       </c>
       <c r="AM8" t="n">
@@ -1599,10 +1674,23 @@
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr"/>
       <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="inlineStr"/>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>散装饼干</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1735,6 +1823,11 @@
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="inlineStr"/>
       <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1867,6 +1960,11 @@
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
       <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1999,6 +2097,11 @@
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr"/>
       <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2131,6 +2234,11 @@
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
       <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2263,6 +2371,11 @@
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
       <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2395,6 +2508,11 @@
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
       <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr"/>
+      <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr"/>
+      <c r="AY14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2527,6 +2645,11 @@
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="inlineStr"/>
       <c r="AT15" t="inlineStr"/>
+      <c r="AU15" t="inlineStr"/>
+      <c r="AV15" t="inlineStr"/>
+      <c r="AW15" t="inlineStr"/>
+      <c r="AX15" t="inlineStr"/>
+      <c r="AY15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2659,6 +2782,11 @@
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="inlineStr"/>
       <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr"/>
+      <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2791,6 +2919,11 @@
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="inlineStr"/>
       <c r="AT17" t="inlineStr"/>
+      <c r="AU17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr"/>
+      <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
+      <c r="AY17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2923,6 +3056,11 @@
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="inlineStr"/>
       <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -3055,6 +3193,11 @@
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="inlineStr"/>
       <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3187,6 +3330,11 @@
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="inlineStr"/>
       <c r="AT20" t="inlineStr"/>
+      <c r="AU20" t="inlineStr"/>
+      <c r="AV20" t="inlineStr"/>
+      <c r="AW20" t="inlineStr"/>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -3319,6 +3467,11 @@
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="inlineStr"/>
       <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr"/>
+      <c r="AW21" t="inlineStr"/>
+      <c r="AX21" t="inlineStr"/>
+      <c r="AY21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3451,6 +3604,11 @@
       <c r="AR22" t="inlineStr"/>
       <c r="AS22" t="inlineStr"/>
       <c r="AT22" t="inlineStr"/>
+      <c r="AU22" t="inlineStr"/>
+      <c r="AV22" t="inlineStr"/>
+      <c r="AW22" t="inlineStr"/>
+      <c r="AX22" t="inlineStr"/>
+      <c r="AY22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -3583,6 +3741,11 @@
       <c r="AR23" t="inlineStr"/>
       <c r="AS23" t="inlineStr"/>
       <c r="AT23" t="inlineStr"/>
+      <c r="AU23" t="inlineStr"/>
+      <c r="AV23" t="inlineStr"/>
+      <c r="AW23" t="inlineStr"/>
+      <c r="AX23" t="inlineStr"/>
+      <c r="AY23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3715,6 +3878,11 @@
       <c r="AR24" t="inlineStr"/>
       <c r="AS24" t="inlineStr"/>
       <c r="AT24" t="inlineStr"/>
+      <c r="AU24" t="inlineStr"/>
+      <c r="AV24" t="inlineStr"/>
+      <c r="AW24" t="inlineStr"/>
+      <c r="AX24" t="inlineStr"/>
+      <c r="AY24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -3847,6 +4015,11 @@
       <c r="AR25" t="inlineStr"/>
       <c r="AS25" t="inlineStr"/>
       <c r="AT25" t="inlineStr"/>
+      <c r="AU25" t="inlineStr"/>
+      <c r="AV25" t="inlineStr"/>
+      <c r="AW25" t="inlineStr"/>
+      <c r="AX25" t="inlineStr"/>
+      <c r="AY25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3979,6 +4152,11 @@
       <c r="AR26" t="inlineStr"/>
       <c r="AS26" t="inlineStr"/>
       <c r="AT26" t="inlineStr"/>
+      <c r="AU26" t="inlineStr"/>
+      <c r="AV26" t="inlineStr"/>
+      <c r="AW26" t="inlineStr"/>
+      <c r="AX26" t="inlineStr"/>
+      <c r="AY26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -4111,6 +4289,11 @@
       <c r="AR27" t="inlineStr"/>
       <c r="AS27" t="inlineStr"/>
       <c r="AT27" t="inlineStr"/>
+      <c r="AU27" t="inlineStr"/>
+      <c r="AV27" t="inlineStr"/>
+      <c r="AW27" t="inlineStr"/>
+      <c r="AX27" t="inlineStr"/>
+      <c r="AY27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -4243,6 +4426,11 @@
       <c r="AR28" t="inlineStr"/>
       <c r="AS28" t="inlineStr"/>
       <c r="AT28" t="inlineStr"/>
+      <c r="AU28" t="inlineStr"/>
+      <c r="AV28" t="inlineStr"/>
+      <c r="AW28" t="inlineStr"/>
+      <c r="AX28" t="inlineStr"/>
+      <c r="AY28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -4375,6 +4563,11 @@
       <c r="AR29" t="inlineStr"/>
       <c r="AS29" t="inlineStr"/>
       <c r="AT29" t="inlineStr"/>
+      <c r="AU29" t="inlineStr"/>
+      <c r="AV29" t="inlineStr"/>
+      <c r="AW29" t="inlineStr"/>
+      <c r="AX29" t="inlineStr"/>
+      <c r="AY29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -4507,6 +4700,11 @@
       <c r="AR30" t="inlineStr"/>
       <c r="AS30" t="inlineStr"/>
       <c r="AT30" t="inlineStr"/>
+      <c r="AU30" t="inlineStr"/>
+      <c r="AV30" t="inlineStr"/>
+      <c r="AW30" t="inlineStr"/>
+      <c r="AX30" t="inlineStr"/>
+      <c r="AY30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -4639,6 +4837,11 @@
       <c r="AR31" t="inlineStr"/>
       <c r="AS31" t="inlineStr"/>
       <c r="AT31" t="inlineStr"/>
+      <c r="AU31" t="inlineStr"/>
+      <c r="AV31" t="inlineStr"/>
+      <c r="AW31" t="inlineStr"/>
+      <c r="AX31" t="inlineStr"/>
+      <c r="AY31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -4771,6 +4974,11 @@
       <c r="AR32" t="inlineStr"/>
       <c r="AS32" t="inlineStr"/>
       <c r="AT32" t="inlineStr"/>
+      <c r="AU32" t="inlineStr"/>
+      <c r="AV32" t="inlineStr"/>
+      <c r="AW32" t="inlineStr"/>
+      <c r="AX32" t="inlineStr"/>
+      <c r="AY32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -4903,6 +5111,11 @@
       <c r="AR33" t="inlineStr"/>
       <c r="AS33" t="inlineStr"/>
       <c r="AT33" t="inlineStr"/>
+      <c r="AU33" t="inlineStr"/>
+      <c r="AV33" t="inlineStr"/>
+      <c r="AW33" t="inlineStr"/>
+      <c r="AX33" t="inlineStr"/>
+      <c r="AY33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -5035,6 +5248,11 @@
       <c r="AR34" t="inlineStr"/>
       <c r="AS34" t="inlineStr"/>
       <c r="AT34" t="inlineStr"/>
+      <c r="AU34" t="inlineStr"/>
+      <c r="AV34" t="inlineStr"/>
+      <c r="AW34" t="inlineStr"/>
+      <c r="AX34" t="inlineStr"/>
+      <c r="AY34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -5167,6 +5385,11 @@
       <c r="AR35" t="inlineStr"/>
       <c r="AS35" t="inlineStr"/>
       <c r="AT35" t="inlineStr"/>
+      <c r="AU35" t="inlineStr"/>
+      <c r="AV35" t="inlineStr"/>
+      <c r="AW35" t="inlineStr"/>
+      <c r="AX35" t="inlineStr"/>
+      <c r="AY35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -5299,6 +5522,11 @@
       <c r="AR36" t="inlineStr"/>
       <c r="AS36" t="inlineStr"/>
       <c r="AT36" t="inlineStr"/>
+      <c r="AU36" t="inlineStr"/>
+      <c r="AV36" t="inlineStr"/>
+      <c r="AW36" t="inlineStr"/>
+      <c r="AX36" t="inlineStr"/>
+      <c r="AY36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -5431,6 +5659,11 @@
       <c r="AR37" t="inlineStr"/>
       <c r="AS37" t="inlineStr"/>
       <c r="AT37" t="inlineStr"/>
+      <c r="AU37" t="inlineStr"/>
+      <c r="AV37" t="inlineStr"/>
+      <c r="AW37" t="inlineStr"/>
+      <c r="AX37" t="inlineStr"/>
+      <c r="AY37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -5563,6 +5796,11 @@
       <c r="AR38" t="inlineStr"/>
       <c r="AS38" t="inlineStr"/>
       <c r="AT38" t="inlineStr"/>
+      <c r="AU38" t="inlineStr"/>
+      <c r="AV38" t="inlineStr"/>
+      <c r="AW38" t="inlineStr"/>
+      <c r="AX38" t="inlineStr"/>
+      <c r="AY38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -5695,6 +5933,11 @@
       <c r="AR39" t="inlineStr"/>
       <c r="AS39" t="inlineStr"/>
       <c r="AT39" t="inlineStr"/>
+      <c r="AU39" t="inlineStr"/>
+      <c r="AV39" t="inlineStr"/>
+      <c r="AW39" t="inlineStr"/>
+      <c r="AX39" t="inlineStr"/>
+      <c r="AY39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -5827,6 +6070,11 @@
       <c r="AR40" t="inlineStr"/>
       <c r="AS40" t="inlineStr"/>
       <c r="AT40" t="inlineStr"/>
+      <c r="AU40" t="inlineStr"/>
+      <c r="AV40" t="inlineStr"/>
+      <c r="AW40" t="inlineStr"/>
+      <c r="AX40" t="inlineStr"/>
+      <c r="AY40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -5959,6 +6207,11 @@
       <c r="AR41" t="inlineStr"/>
       <c r="AS41" t="inlineStr"/>
       <c r="AT41" t="inlineStr"/>
+      <c r="AU41" t="inlineStr"/>
+      <c r="AV41" t="inlineStr"/>
+      <c r="AW41" t="inlineStr"/>
+      <c r="AX41" t="inlineStr"/>
+      <c r="AY41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -6091,6 +6344,11 @@
       <c r="AR42" t="inlineStr"/>
       <c r="AS42" t="inlineStr"/>
       <c r="AT42" t="inlineStr"/>
+      <c r="AU42" t="inlineStr"/>
+      <c r="AV42" t="inlineStr"/>
+      <c r="AW42" t="inlineStr"/>
+      <c r="AX42" t="inlineStr"/>
+      <c r="AY42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -6223,6 +6481,11 @@
       <c r="AR43" t="inlineStr"/>
       <c r="AS43" t="inlineStr"/>
       <c r="AT43" t="inlineStr"/>
+      <c r="AU43" t="inlineStr"/>
+      <c r="AV43" t="inlineStr"/>
+      <c r="AW43" t="inlineStr"/>
+      <c r="AX43" t="inlineStr"/>
+      <c r="AY43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -6355,6 +6618,11 @@
       <c r="AR44" t="inlineStr"/>
       <c r="AS44" t="inlineStr"/>
       <c r="AT44" t="inlineStr"/>
+      <c r="AU44" t="inlineStr"/>
+      <c r="AV44" t="inlineStr"/>
+      <c r="AW44" t="inlineStr"/>
+      <c r="AX44" t="inlineStr"/>
+      <c r="AY44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -6487,6 +6755,11 @@
       <c r="AR45" t="inlineStr"/>
       <c r="AS45" t="inlineStr"/>
       <c r="AT45" t="inlineStr"/>
+      <c r="AU45" t="inlineStr"/>
+      <c r="AV45" t="inlineStr"/>
+      <c r="AW45" t="inlineStr"/>
+      <c r="AX45" t="inlineStr"/>
+      <c r="AY45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -6619,6 +6892,11 @@
       <c r="AR46" t="inlineStr"/>
       <c r="AS46" t="inlineStr"/>
       <c r="AT46" t="inlineStr"/>
+      <c r="AU46" t="inlineStr"/>
+      <c r="AV46" t="inlineStr"/>
+      <c r="AW46" t="inlineStr"/>
+      <c r="AX46" t="inlineStr"/>
+      <c r="AY46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -6751,6 +7029,11 @@
       <c r="AR47" t="inlineStr"/>
       <c r="AS47" t="inlineStr"/>
       <c r="AT47" t="inlineStr"/>
+      <c r="AU47" t="inlineStr"/>
+      <c r="AV47" t="inlineStr"/>
+      <c r="AW47" t="inlineStr"/>
+      <c r="AX47" t="inlineStr"/>
+      <c r="AY47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -6883,6 +7166,11 @@
       <c r="AR48" t="inlineStr"/>
       <c r="AS48" t="inlineStr"/>
       <c r="AT48" t="inlineStr"/>
+      <c r="AU48" t="inlineStr"/>
+      <c r="AV48" t="inlineStr"/>
+      <c r="AW48" t="inlineStr"/>
+      <c r="AX48" t="inlineStr"/>
+      <c r="AY48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -7015,6 +7303,11 @@
       <c r="AR49" t="inlineStr"/>
       <c r="AS49" t="inlineStr"/>
       <c r="AT49" t="inlineStr"/>
+      <c r="AU49" t="inlineStr"/>
+      <c r="AV49" t="inlineStr"/>
+      <c r="AW49" t="inlineStr"/>
+      <c r="AX49" t="inlineStr"/>
+      <c r="AY49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -7147,6 +7440,11 @@
       <c r="AR50" t="inlineStr"/>
       <c r="AS50" t="inlineStr"/>
       <c r="AT50" t="inlineStr"/>
+      <c r="AU50" t="inlineStr"/>
+      <c r="AV50" t="inlineStr"/>
+      <c r="AW50" t="inlineStr"/>
+      <c r="AX50" t="inlineStr"/>
+      <c r="AY50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -7279,6 +7577,11 @@
       <c r="AR51" t="inlineStr"/>
       <c r="AS51" t="inlineStr"/>
       <c r="AT51" t="inlineStr"/>
+      <c r="AU51" t="inlineStr"/>
+      <c r="AV51" t="inlineStr"/>
+      <c r="AW51" t="inlineStr"/>
+      <c r="AX51" t="inlineStr"/>
+      <c r="AY51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -7411,6 +7714,11 @@
       <c r="AR52" t="inlineStr"/>
       <c r="AS52" t="inlineStr"/>
       <c r="AT52" t="inlineStr"/>
+      <c r="AU52" t="inlineStr"/>
+      <c r="AV52" t="inlineStr"/>
+      <c r="AW52" t="inlineStr"/>
+      <c r="AX52" t="inlineStr"/>
+      <c r="AY52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -7543,6 +7851,11 @@
       <c r="AR53" t="inlineStr"/>
       <c r="AS53" t="inlineStr"/>
       <c r="AT53" t="inlineStr"/>
+      <c r="AU53" t="inlineStr"/>
+      <c r="AV53" t="inlineStr"/>
+      <c r="AW53" t="inlineStr"/>
+      <c r="AX53" t="inlineStr"/>
+      <c r="AY53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -7675,6 +7988,11 @@
       <c r="AR54" t="inlineStr"/>
       <c r="AS54" t="inlineStr"/>
       <c r="AT54" t="inlineStr"/>
+      <c r="AU54" t="inlineStr"/>
+      <c r="AV54" t="inlineStr"/>
+      <c r="AW54" t="inlineStr"/>
+      <c r="AX54" t="inlineStr"/>
+      <c r="AY54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -7807,6 +8125,11 @@
       <c r="AR55" t="inlineStr"/>
       <c r="AS55" t="inlineStr"/>
       <c r="AT55" t="inlineStr"/>
+      <c r="AU55" t="inlineStr"/>
+      <c r="AV55" t="inlineStr"/>
+      <c r="AW55" t="inlineStr"/>
+      <c r="AX55" t="inlineStr"/>
+      <c r="AY55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -7939,6 +8262,11 @@
       <c r="AR56" t="inlineStr"/>
       <c r="AS56" t="inlineStr"/>
       <c r="AT56" t="inlineStr"/>
+      <c r="AU56" t="inlineStr"/>
+      <c r="AV56" t="inlineStr"/>
+      <c r="AW56" t="inlineStr"/>
+      <c r="AX56" t="inlineStr"/>
+      <c r="AY56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -8071,6 +8399,11 @@
       <c r="AR57" t="inlineStr"/>
       <c r="AS57" t="inlineStr"/>
       <c r="AT57" t="inlineStr"/>
+      <c r="AU57" t="inlineStr"/>
+      <c r="AV57" t="inlineStr"/>
+      <c r="AW57" t="inlineStr"/>
+      <c r="AX57" t="inlineStr"/>
+      <c r="AY57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -8203,6 +8536,11 @@
       <c r="AR58" t="inlineStr"/>
       <c r="AS58" t="inlineStr"/>
       <c r="AT58" t="inlineStr"/>
+      <c r="AU58" t="inlineStr"/>
+      <c r="AV58" t="inlineStr"/>
+      <c r="AW58" t="inlineStr"/>
+      <c r="AX58" t="inlineStr"/>
+      <c r="AY58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -8335,6 +8673,11 @@
       <c r="AR59" t="inlineStr"/>
       <c r="AS59" t="inlineStr"/>
       <c r="AT59" t="inlineStr"/>
+      <c r="AU59" t="inlineStr"/>
+      <c r="AV59" t="inlineStr"/>
+      <c r="AW59" t="inlineStr"/>
+      <c r="AX59" t="inlineStr"/>
+      <c r="AY59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -8467,6 +8810,11 @@
       <c r="AR60" t="inlineStr"/>
       <c r="AS60" t="inlineStr"/>
       <c r="AT60" t="inlineStr"/>
+      <c r="AU60" t="inlineStr"/>
+      <c r="AV60" t="inlineStr"/>
+      <c r="AW60" t="inlineStr"/>
+      <c r="AX60" t="inlineStr"/>
+      <c r="AY60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -8599,6 +8947,11 @@
       <c r="AR61" t="inlineStr"/>
       <c r="AS61" t="inlineStr"/>
       <c r="AT61" t="inlineStr"/>
+      <c r="AU61" t="inlineStr"/>
+      <c r="AV61" t="inlineStr"/>
+      <c r="AW61" t="inlineStr"/>
+      <c r="AX61" t="inlineStr"/>
+      <c r="AY61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -8731,6 +9084,11 @@
       <c r="AR62" t="inlineStr"/>
       <c r="AS62" t="inlineStr"/>
       <c r="AT62" t="inlineStr"/>
+      <c r="AU62" t="inlineStr"/>
+      <c r="AV62" t="inlineStr"/>
+      <c r="AW62" t="inlineStr"/>
+      <c r="AX62" t="inlineStr"/>
+      <c r="AY62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -8863,6 +9221,11 @@
       <c r="AR63" t="inlineStr"/>
       <c r="AS63" t="inlineStr"/>
       <c r="AT63" t="inlineStr"/>
+      <c r="AU63" t="inlineStr"/>
+      <c r="AV63" t="inlineStr"/>
+      <c r="AW63" t="inlineStr"/>
+      <c r="AX63" t="inlineStr"/>
+      <c r="AY63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -8995,6 +9358,11 @@
       <c r="AR64" t="inlineStr"/>
       <c r="AS64" t="inlineStr"/>
       <c r="AT64" t="inlineStr"/>
+      <c r="AU64" t="inlineStr"/>
+      <c r="AV64" t="inlineStr"/>
+      <c r="AW64" t="inlineStr"/>
+      <c r="AX64" t="inlineStr"/>
+      <c r="AY64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -9127,6 +9495,11 @@
       <c r="AR65" t="inlineStr"/>
       <c r="AS65" t="inlineStr"/>
       <c r="AT65" t="inlineStr"/>
+      <c r="AU65" t="inlineStr"/>
+      <c r="AV65" t="inlineStr"/>
+      <c r="AW65" t="inlineStr"/>
+      <c r="AX65" t="inlineStr"/>
+      <c r="AY65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -9259,6 +9632,11 @@
       <c r="AR66" t="inlineStr"/>
       <c r="AS66" t="inlineStr"/>
       <c r="AT66" t="inlineStr"/>
+      <c r="AU66" t="inlineStr"/>
+      <c r="AV66" t="inlineStr"/>
+      <c r="AW66" t="inlineStr"/>
+      <c r="AX66" t="inlineStr"/>
+      <c r="AY66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -9391,6 +9769,11 @@
       <c r="AR67" t="inlineStr"/>
       <c r="AS67" t="inlineStr"/>
       <c r="AT67" t="inlineStr"/>
+      <c r="AU67" t="inlineStr"/>
+      <c r="AV67" t="inlineStr"/>
+      <c r="AW67" t="inlineStr"/>
+      <c r="AX67" t="inlineStr"/>
+      <c r="AY67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -9523,6 +9906,11 @@
       <c r="AR68" t="inlineStr"/>
       <c r="AS68" t="inlineStr"/>
       <c r="AT68" t="inlineStr"/>
+      <c r="AU68" t="inlineStr"/>
+      <c r="AV68" t="inlineStr"/>
+      <c r="AW68" t="inlineStr"/>
+      <c r="AX68" t="inlineStr"/>
+      <c r="AY68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -9655,6 +10043,11 @@
       <c r="AR69" t="inlineStr"/>
       <c r="AS69" t="inlineStr"/>
       <c r="AT69" t="inlineStr"/>
+      <c r="AU69" t="inlineStr"/>
+      <c r="AV69" t="inlineStr"/>
+      <c r="AW69" t="inlineStr"/>
+      <c r="AX69" t="inlineStr"/>
+      <c r="AY69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -9787,6 +10180,11 @@
       <c r="AR70" t="inlineStr"/>
       <c r="AS70" t="inlineStr"/>
       <c r="AT70" t="inlineStr"/>
+      <c r="AU70" t="inlineStr"/>
+      <c r="AV70" t="inlineStr"/>
+      <c r="AW70" t="inlineStr"/>
+      <c r="AX70" t="inlineStr"/>
+      <c r="AY70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -9919,6 +10317,11 @@
       <c r="AR71" t="inlineStr"/>
       <c r="AS71" t="inlineStr"/>
       <c r="AT71" t="inlineStr"/>
+      <c r="AU71" t="inlineStr"/>
+      <c r="AV71" t="inlineStr"/>
+      <c r="AW71" t="inlineStr"/>
+      <c r="AX71" t="inlineStr"/>
+      <c r="AY71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10051,6 +10454,11 @@
       <c r="AR72" t="inlineStr"/>
       <c r="AS72" t="inlineStr"/>
       <c r="AT72" t="inlineStr"/>
+      <c r="AU72" t="inlineStr"/>
+      <c r="AV72" t="inlineStr"/>
+      <c r="AW72" t="inlineStr"/>
+      <c r="AX72" t="inlineStr"/>
+      <c r="AY72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -10183,6 +10591,11 @@
       <c r="AR73" t="inlineStr"/>
       <c r="AS73" t="inlineStr"/>
       <c r="AT73" t="inlineStr"/>
+      <c r="AU73" t="inlineStr"/>
+      <c r="AV73" t="inlineStr"/>
+      <c r="AW73" t="inlineStr"/>
+      <c r="AX73" t="inlineStr"/>
+      <c r="AY73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10315,6 +10728,11 @@
       <c r="AR74" t="inlineStr"/>
       <c r="AS74" t="inlineStr"/>
       <c r="AT74" t="inlineStr"/>
+      <c r="AU74" t="inlineStr"/>
+      <c r="AV74" t="inlineStr"/>
+      <c r="AW74" t="inlineStr"/>
+      <c r="AX74" t="inlineStr"/>
+      <c r="AY74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10447,6 +10865,11 @@
       <c r="AR75" t="inlineStr"/>
       <c r="AS75" t="inlineStr"/>
       <c r="AT75" t="inlineStr"/>
+      <c r="AU75" t="inlineStr"/>
+      <c r="AV75" t="inlineStr"/>
+      <c r="AW75" t="inlineStr"/>
+      <c r="AX75" t="inlineStr"/>
+      <c r="AY75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10579,6 +11002,11 @@
       <c r="AR76" t="inlineStr"/>
       <c r="AS76" t="inlineStr"/>
       <c r="AT76" t="inlineStr"/>
+      <c r="AU76" t="inlineStr"/>
+      <c r="AV76" t="inlineStr"/>
+      <c r="AW76" t="inlineStr"/>
+      <c r="AX76" t="inlineStr"/>
+      <c r="AY76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -10711,6 +11139,11 @@
       <c r="AR77" t="inlineStr"/>
       <c r="AS77" t="inlineStr"/>
       <c r="AT77" t="inlineStr"/>
+      <c r="AU77" t="inlineStr"/>
+      <c r="AV77" t="inlineStr"/>
+      <c r="AW77" t="inlineStr"/>
+      <c r="AX77" t="inlineStr"/>
+      <c r="AY77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -10843,6 +11276,11 @@
       <c r="AR78" t="inlineStr"/>
       <c r="AS78" t="inlineStr"/>
       <c r="AT78" t="inlineStr"/>
+      <c r="AU78" t="inlineStr"/>
+      <c r="AV78" t="inlineStr"/>
+      <c r="AW78" t="inlineStr"/>
+      <c r="AX78" t="inlineStr"/>
+      <c r="AY78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -10975,6 +11413,11 @@
       <c r="AR79" t="inlineStr"/>
       <c r="AS79" t="inlineStr"/>
       <c r="AT79" t="inlineStr"/>
+      <c r="AU79" t="inlineStr"/>
+      <c r="AV79" t="inlineStr"/>
+      <c r="AW79" t="inlineStr"/>
+      <c r="AX79" t="inlineStr"/>
+      <c r="AY79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -11107,6 +11550,11 @@
       <c r="AR80" t="inlineStr"/>
       <c r="AS80" t="inlineStr"/>
       <c r="AT80" t="inlineStr"/>
+      <c r="AU80" t="inlineStr"/>
+      <c r="AV80" t="inlineStr"/>
+      <c r="AW80" t="inlineStr"/>
+      <c r="AX80" t="inlineStr"/>
+      <c r="AY80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -11235,6 +11683,11 @@
       <c r="AR81" t="inlineStr"/>
       <c r="AS81" t="inlineStr"/>
       <c r="AT81" t="inlineStr"/>
+      <c r="AU81" t="inlineStr"/>
+      <c r="AV81" t="inlineStr"/>
+      <c r="AW81" t="inlineStr"/>
+      <c r="AX81" t="inlineStr"/>
+      <c r="AY81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -11367,6 +11820,11 @@
       <c r="AR82" t="inlineStr"/>
       <c r="AS82" t="inlineStr"/>
       <c r="AT82" t="inlineStr"/>
+      <c r="AU82" t="inlineStr"/>
+      <c r="AV82" t="inlineStr"/>
+      <c r="AW82" t="inlineStr"/>
+      <c r="AX82" t="inlineStr"/>
+      <c r="AY82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -11499,6 +11957,11 @@
       <c r="AR83" t="inlineStr"/>
       <c r="AS83" t="inlineStr"/>
       <c r="AT83" t="inlineStr"/>
+      <c r="AU83" t="inlineStr"/>
+      <c r="AV83" t="inlineStr"/>
+      <c r="AW83" t="inlineStr"/>
+      <c r="AX83" t="inlineStr"/>
+      <c r="AY83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -11631,6 +12094,11 @@
       <c r="AR84" t="inlineStr"/>
       <c r="AS84" t="inlineStr"/>
       <c r="AT84" t="inlineStr"/>
+      <c r="AU84" t="inlineStr"/>
+      <c r="AV84" t="inlineStr"/>
+      <c r="AW84" t="inlineStr"/>
+      <c r="AX84" t="inlineStr"/>
+      <c r="AY84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -11763,6 +12231,11 @@
       <c r="AR85" t="inlineStr"/>
       <c r="AS85" t="inlineStr"/>
       <c r="AT85" t="inlineStr"/>
+      <c r="AU85" t="inlineStr"/>
+      <c r="AV85" t="inlineStr"/>
+      <c r="AW85" t="inlineStr"/>
+      <c r="AX85" t="inlineStr"/>
+      <c r="AY85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -11895,6 +12368,11 @@
       <c r="AR86" t="inlineStr"/>
       <c r="AS86" t="inlineStr"/>
       <c r="AT86" t="inlineStr"/>
+      <c r="AU86" t="inlineStr"/>
+      <c r="AV86" t="inlineStr"/>
+      <c r="AW86" t="inlineStr"/>
+      <c r="AX86" t="inlineStr"/>
+      <c r="AY86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -12027,6 +12505,11 @@
       <c r="AR87" t="inlineStr"/>
       <c r="AS87" t="inlineStr"/>
       <c r="AT87" t="inlineStr"/>
+      <c r="AU87" t="inlineStr"/>
+      <c r="AV87" t="inlineStr"/>
+      <c r="AW87" t="inlineStr"/>
+      <c r="AX87" t="inlineStr"/>
+      <c r="AY87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -12159,6 +12642,11 @@
       <c r="AR88" t="inlineStr"/>
       <c r="AS88" t="inlineStr"/>
       <c r="AT88" t="inlineStr"/>
+      <c r="AU88" t="inlineStr"/>
+      <c r="AV88" t="inlineStr"/>
+      <c r="AW88" t="inlineStr"/>
+      <c r="AX88" t="inlineStr"/>
+      <c r="AY88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -12291,6 +12779,11 @@
       <c r="AR89" t="inlineStr"/>
       <c r="AS89" t="inlineStr"/>
       <c r="AT89" t="inlineStr"/>
+      <c r="AU89" t="inlineStr"/>
+      <c r="AV89" t="inlineStr"/>
+      <c r="AW89" t="inlineStr"/>
+      <c r="AX89" t="inlineStr"/>
+      <c r="AY89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -12423,6 +12916,11 @@
       <c r="AR90" t="inlineStr"/>
       <c r="AS90" t="inlineStr"/>
       <c r="AT90" t="inlineStr"/>
+      <c r="AU90" t="inlineStr"/>
+      <c r="AV90" t="inlineStr"/>
+      <c r="AW90" t="inlineStr"/>
+      <c r="AX90" t="inlineStr"/>
+      <c r="AY90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -12555,6 +13053,11 @@
       <c r="AR91" t="inlineStr"/>
       <c r="AS91" t="inlineStr"/>
       <c r="AT91" t="inlineStr"/>
+      <c r="AU91" t="inlineStr"/>
+      <c r="AV91" t="inlineStr"/>
+      <c r="AW91" t="inlineStr"/>
+      <c r="AX91" t="inlineStr"/>
+      <c r="AY91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -12687,6 +13190,11 @@
       <c r="AR92" t="inlineStr"/>
       <c r="AS92" t="inlineStr"/>
       <c r="AT92" t="inlineStr"/>
+      <c r="AU92" t="inlineStr"/>
+      <c r="AV92" t="inlineStr"/>
+      <c r="AW92" t="inlineStr"/>
+      <c r="AX92" t="inlineStr"/>
+      <c r="AY92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -12819,6 +13327,11 @@
       <c r="AR93" t="inlineStr"/>
       <c r="AS93" t="inlineStr"/>
       <c r="AT93" t="inlineStr"/>
+      <c r="AU93" t="inlineStr"/>
+      <c r="AV93" t="inlineStr"/>
+      <c r="AW93" t="inlineStr"/>
+      <c r="AX93" t="inlineStr"/>
+      <c r="AY93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -12951,6 +13464,11 @@
       <c r="AR94" t="inlineStr"/>
       <c r="AS94" t="inlineStr"/>
       <c r="AT94" t="inlineStr"/>
+      <c r="AU94" t="inlineStr"/>
+      <c r="AV94" t="inlineStr"/>
+      <c r="AW94" t="inlineStr"/>
+      <c r="AX94" t="inlineStr"/>
+      <c r="AY94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -13083,6 +13601,11 @@
       <c r="AR95" t="inlineStr"/>
       <c r="AS95" t="inlineStr"/>
       <c r="AT95" t="inlineStr"/>
+      <c r="AU95" t="inlineStr"/>
+      <c r="AV95" t="inlineStr"/>
+      <c r="AW95" t="inlineStr"/>
+      <c r="AX95" t="inlineStr"/>
+      <c r="AY95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -13215,6 +13738,11 @@
       <c r="AR96" t="inlineStr"/>
       <c r="AS96" t="inlineStr"/>
       <c r="AT96" t="inlineStr"/>
+      <c r="AU96" t="inlineStr"/>
+      <c r="AV96" t="inlineStr"/>
+      <c r="AW96" t="inlineStr"/>
+      <c r="AX96" t="inlineStr"/>
+      <c r="AY96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -13347,6 +13875,11 @@
       <c r="AR97" t="inlineStr"/>
       <c r="AS97" t="inlineStr"/>
       <c r="AT97" t="inlineStr"/>
+      <c r="AU97" t="inlineStr"/>
+      <c r="AV97" t="inlineStr"/>
+      <c r="AW97" t="inlineStr"/>
+      <c r="AX97" t="inlineStr"/>
+      <c r="AY97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -13479,6 +14012,11 @@
       <c r="AR98" t="inlineStr"/>
       <c r="AS98" t="inlineStr"/>
       <c r="AT98" t="inlineStr"/>
+      <c r="AU98" t="inlineStr"/>
+      <c r="AV98" t="inlineStr"/>
+      <c r="AW98" t="inlineStr"/>
+      <c r="AX98" t="inlineStr"/>
+      <c r="AY98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -13611,6 +14149,11 @@
       <c r="AR99" t="inlineStr"/>
       <c r="AS99" t="inlineStr"/>
       <c r="AT99" t="inlineStr"/>
+      <c r="AU99" t="inlineStr"/>
+      <c r="AV99" t="inlineStr"/>
+      <c r="AW99" t="inlineStr"/>
+      <c r="AX99" t="inlineStr"/>
+      <c r="AY99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -13743,6 +14286,11 @@
       <c r="AR100" t="inlineStr"/>
       <c r="AS100" t="inlineStr"/>
       <c r="AT100" t="inlineStr"/>
+      <c r="AU100" t="inlineStr"/>
+      <c r="AV100" t="inlineStr"/>
+      <c r="AW100" t="inlineStr"/>
+      <c r="AX100" t="inlineStr"/>
+      <c r="AY100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -13875,6 +14423,11 @@
       <c r="AR101" t="inlineStr"/>
       <c r="AS101" t="inlineStr"/>
       <c r="AT101" t="inlineStr"/>
+      <c r="AU101" t="inlineStr"/>
+      <c r="AV101" t="inlineStr"/>
+      <c r="AW101" t="inlineStr"/>
+      <c r="AX101" t="inlineStr"/>
+      <c r="AY101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -14007,6 +14560,11 @@
       <c r="AR102" t="inlineStr"/>
       <c r="AS102" t="inlineStr"/>
       <c r="AT102" t="inlineStr"/>
+      <c r="AU102" t="inlineStr"/>
+      <c r="AV102" t="inlineStr"/>
+      <c r="AW102" t="inlineStr"/>
+      <c r="AX102" t="inlineStr"/>
+      <c r="AY102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -14139,6 +14697,11 @@
       <c r="AR103" t="inlineStr"/>
       <c r="AS103" t="inlineStr"/>
       <c r="AT103" t="inlineStr"/>
+      <c r="AU103" t="inlineStr"/>
+      <c r="AV103" t="inlineStr"/>
+      <c r="AW103" t="inlineStr"/>
+      <c r="AX103" t="inlineStr"/>
+      <c r="AY103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -14271,6 +14834,11 @@
       <c r="AR104" t="inlineStr"/>
       <c r="AS104" t="inlineStr"/>
       <c r="AT104" t="inlineStr"/>
+      <c r="AU104" t="inlineStr"/>
+      <c r="AV104" t="inlineStr"/>
+      <c r="AW104" t="inlineStr"/>
+      <c r="AX104" t="inlineStr"/>
+      <c r="AY104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -14403,6 +14971,11 @@
       <c r="AR105" t="inlineStr"/>
       <c r="AS105" t="inlineStr"/>
       <c r="AT105" t="inlineStr"/>
+      <c r="AU105" t="inlineStr"/>
+      <c r="AV105" t="inlineStr"/>
+      <c r="AW105" t="inlineStr"/>
+      <c r="AX105" t="inlineStr"/>
+      <c r="AY105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -14535,6 +15108,11 @@
       <c r="AR106" t="inlineStr"/>
       <c r="AS106" t="inlineStr"/>
       <c r="AT106" t="inlineStr"/>
+      <c r="AU106" t="inlineStr"/>
+      <c r="AV106" t="inlineStr"/>
+      <c r="AW106" t="inlineStr"/>
+      <c r="AX106" t="inlineStr"/>
+      <c r="AY106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -14667,6 +15245,11 @@
       <c r="AR107" t="inlineStr"/>
       <c r="AS107" t="inlineStr"/>
       <c r="AT107" t="inlineStr"/>
+      <c r="AU107" t="inlineStr"/>
+      <c r="AV107" t="inlineStr"/>
+      <c r="AW107" t="inlineStr"/>
+      <c r="AX107" t="inlineStr"/>
+      <c r="AY107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -14795,6 +15378,11 @@
       <c r="AR108" t="inlineStr"/>
       <c r="AS108" t="inlineStr"/>
       <c r="AT108" t="inlineStr"/>
+      <c r="AU108" t="inlineStr"/>
+      <c r="AV108" t="inlineStr"/>
+      <c r="AW108" t="inlineStr"/>
+      <c r="AX108" t="inlineStr"/>
+      <c r="AY108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -14927,6 +15515,11 @@
       <c r="AR109" t="inlineStr"/>
       <c r="AS109" t="inlineStr"/>
       <c r="AT109" t="inlineStr"/>
+      <c r="AU109" t="inlineStr"/>
+      <c r="AV109" t="inlineStr"/>
+      <c r="AW109" t="inlineStr"/>
+      <c r="AX109" t="inlineStr"/>
+      <c r="AY109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -15059,6 +15652,11 @@
       <c r="AR110" t="inlineStr"/>
       <c r="AS110" t="inlineStr"/>
       <c r="AT110" t="inlineStr"/>
+      <c r="AU110" t="inlineStr"/>
+      <c r="AV110" t="inlineStr"/>
+      <c r="AW110" t="inlineStr"/>
+      <c r="AX110" t="inlineStr"/>
+      <c r="AY110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -15187,6 +15785,11 @@
       <c r="AR111" t="inlineStr"/>
       <c r="AS111" t="inlineStr"/>
       <c r="AT111" t="inlineStr"/>
+      <c r="AU111" t="inlineStr"/>
+      <c r="AV111" t="inlineStr"/>
+      <c r="AW111" t="inlineStr"/>
+      <c r="AX111" t="inlineStr"/>
+      <c r="AY111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -15315,6 +15918,11 @@
       <c r="AR112" t="inlineStr"/>
       <c r="AS112" t="inlineStr"/>
       <c r="AT112" t="inlineStr"/>
+      <c r="AU112" t="inlineStr"/>
+      <c r="AV112" t="inlineStr"/>
+      <c r="AW112" t="inlineStr"/>
+      <c r="AX112" t="inlineStr"/>
+      <c r="AY112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -15447,6 +16055,11 @@
       <c r="AR113" t="inlineStr"/>
       <c r="AS113" t="inlineStr"/>
       <c r="AT113" t="inlineStr"/>
+      <c r="AU113" t="inlineStr"/>
+      <c r="AV113" t="inlineStr"/>
+      <c r="AW113" t="inlineStr"/>
+      <c r="AX113" t="inlineStr"/>
+      <c r="AY113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -15579,6 +16192,11 @@
       <c r="AR114" t="inlineStr"/>
       <c r="AS114" t="inlineStr"/>
       <c r="AT114" t="inlineStr"/>
+      <c r="AU114" t="inlineStr"/>
+      <c r="AV114" t="inlineStr"/>
+      <c r="AW114" t="inlineStr"/>
+      <c r="AX114" t="inlineStr"/>
+      <c r="AY114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -15711,6 +16329,11 @@
       <c r="AR115" t="inlineStr"/>
       <c r="AS115" t="inlineStr"/>
       <c r="AT115" t="inlineStr"/>
+      <c r="AU115" t="inlineStr"/>
+      <c r="AV115" t="inlineStr"/>
+      <c r="AW115" t="inlineStr"/>
+      <c r="AX115" t="inlineStr"/>
+      <c r="AY115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -15843,6 +16466,11 @@
       <c r="AR116" t="inlineStr"/>
       <c r="AS116" t="inlineStr"/>
       <c r="AT116" t="inlineStr"/>
+      <c r="AU116" t="inlineStr"/>
+      <c r="AV116" t="inlineStr"/>
+      <c r="AW116" t="inlineStr"/>
+      <c r="AX116" t="inlineStr"/>
+      <c r="AY116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -15975,6 +16603,11 @@
       <c r="AR117" t="inlineStr"/>
       <c r="AS117" t="inlineStr"/>
       <c r="AT117" t="inlineStr"/>
+      <c r="AU117" t="inlineStr"/>
+      <c r="AV117" t="inlineStr"/>
+      <c r="AW117" t="inlineStr"/>
+      <c r="AX117" t="inlineStr"/>
+      <c r="AY117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -16107,6 +16740,11 @@
       <c r="AR118" t="inlineStr"/>
       <c r="AS118" t="inlineStr"/>
       <c r="AT118" t="inlineStr"/>
+      <c r="AU118" t="inlineStr"/>
+      <c r="AV118" t="inlineStr"/>
+      <c r="AW118" t="inlineStr"/>
+      <c r="AX118" t="inlineStr"/>
+      <c r="AY118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -16239,6 +16877,11 @@
       <c r="AR119" t="inlineStr"/>
       <c r="AS119" t="inlineStr"/>
       <c r="AT119" t="inlineStr"/>
+      <c r="AU119" t="inlineStr"/>
+      <c r="AV119" t="inlineStr"/>
+      <c r="AW119" t="inlineStr"/>
+      <c r="AX119" t="inlineStr"/>
+      <c r="AY119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -16371,6 +17014,11 @@
       <c r="AR120" t="inlineStr"/>
       <c r="AS120" t="inlineStr"/>
       <c r="AT120" t="inlineStr"/>
+      <c r="AU120" t="inlineStr"/>
+      <c r="AV120" t="inlineStr"/>
+      <c r="AW120" t="inlineStr"/>
+      <c r="AX120" t="inlineStr"/>
+      <c r="AY120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -16499,6 +17147,11 @@
       <c r="AR121" t="inlineStr"/>
       <c r="AS121" t="inlineStr"/>
       <c r="AT121" t="inlineStr"/>
+      <c r="AU121" t="inlineStr"/>
+      <c r="AV121" t="inlineStr"/>
+      <c r="AW121" t="inlineStr"/>
+      <c r="AX121" t="inlineStr"/>
+      <c r="AY121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -16627,6 +17280,11 @@
       <c r="AR122" t="inlineStr"/>
       <c r="AS122" t="inlineStr"/>
       <c r="AT122" t="inlineStr"/>
+      <c r="AU122" t="inlineStr"/>
+      <c r="AV122" t="inlineStr"/>
+      <c r="AW122" t="inlineStr"/>
+      <c r="AX122" t="inlineStr"/>
+      <c r="AY122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -16755,6 +17413,11 @@
       <c r="AR123" t="inlineStr"/>
       <c r="AS123" t="inlineStr"/>
       <c r="AT123" t="inlineStr"/>
+      <c r="AU123" t="inlineStr"/>
+      <c r="AV123" t="inlineStr"/>
+      <c r="AW123" t="inlineStr"/>
+      <c r="AX123" t="inlineStr"/>
+      <c r="AY123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -16883,6 +17546,11 @@
       <c r="AR124" t="inlineStr"/>
       <c r="AS124" t="inlineStr"/>
       <c r="AT124" t="inlineStr"/>
+      <c r="AU124" t="inlineStr"/>
+      <c r="AV124" t="inlineStr"/>
+      <c r="AW124" t="inlineStr"/>
+      <c r="AX124" t="inlineStr"/>
+      <c r="AY124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -17011,6 +17679,11 @@
       <c r="AR125" t="inlineStr"/>
       <c r="AS125" t="inlineStr"/>
       <c r="AT125" t="inlineStr"/>
+      <c r="AU125" t="inlineStr"/>
+      <c r="AV125" t="inlineStr"/>
+      <c r="AW125" t="inlineStr"/>
+      <c r="AX125" t="inlineStr"/>
+      <c r="AY125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -17139,6 +17812,11 @@
       <c r="AR126" t="inlineStr"/>
       <c r="AS126" t="inlineStr"/>
       <c r="AT126" t="inlineStr"/>
+      <c r="AU126" t="inlineStr"/>
+      <c r="AV126" t="inlineStr"/>
+      <c r="AW126" t="inlineStr"/>
+      <c r="AX126" t="inlineStr"/>
+      <c r="AY126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -17267,6 +17945,11 @@
       <c r="AR127" t="inlineStr"/>
       <c r="AS127" t="inlineStr"/>
       <c r="AT127" t="inlineStr"/>
+      <c r="AU127" t="inlineStr"/>
+      <c r="AV127" t="inlineStr"/>
+      <c r="AW127" t="inlineStr"/>
+      <c r="AX127" t="inlineStr"/>
+      <c r="AY127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -17399,6 +18082,11 @@
       <c r="AR128" t="inlineStr"/>
       <c r="AS128" t="inlineStr"/>
       <c r="AT128" t="inlineStr"/>
+      <c r="AU128" t="inlineStr"/>
+      <c r="AV128" t="inlineStr"/>
+      <c r="AW128" t="inlineStr"/>
+      <c r="AX128" t="inlineStr"/>
+      <c r="AY128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -17531,6 +18219,11 @@
       <c r="AR129" t="inlineStr"/>
       <c r="AS129" t="inlineStr"/>
       <c r="AT129" t="inlineStr"/>
+      <c r="AU129" t="inlineStr"/>
+      <c r="AV129" t="inlineStr"/>
+      <c r="AW129" t="inlineStr"/>
+      <c r="AX129" t="inlineStr"/>
+      <c r="AY129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -17663,6 +18356,11 @@
       <c r="AR130" t="inlineStr"/>
       <c r="AS130" t="inlineStr"/>
       <c r="AT130" t="inlineStr"/>
+      <c r="AU130" t="inlineStr"/>
+      <c r="AV130" t="inlineStr"/>
+      <c r="AW130" t="inlineStr"/>
+      <c r="AX130" t="inlineStr"/>
+      <c r="AY130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -17795,6 +18493,11 @@
       <c r="AR131" t="inlineStr"/>
       <c r="AS131" t="inlineStr"/>
       <c r="AT131" t="inlineStr"/>
+      <c r="AU131" t="inlineStr"/>
+      <c r="AV131" t="inlineStr"/>
+      <c r="AW131" t="inlineStr"/>
+      <c r="AX131" t="inlineStr"/>
+      <c r="AY131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -17927,6 +18630,11 @@
       <c r="AR132" t="inlineStr"/>
       <c r="AS132" t="inlineStr"/>
       <c r="AT132" t="inlineStr"/>
+      <c r="AU132" t="inlineStr"/>
+      <c r="AV132" t="inlineStr"/>
+      <c r="AW132" t="inlineStr"/>
+      <c r="AX132" t="inlineStr"/>
+      <c r="AY132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -18059,6 +18767,11 @@
       <c r="AR133" t="inlineStr"/>
       <c r="AS133" t="inlineStr"/>
       <c r="AT133" t="inlineStr"/>
+      <c r="AU133" t="inlineStr"/>
+      <c r="AV133" t="inlineStr"/>
+      <c r="AW133" t="inlineStr"/>
+      <c r="AX133" t="inlineStr"/>
+      <c r="AY133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -18191,6 +18904,11 @@
       <c r="AR134" t="inlineStr"/>
       <c r="AS134" t="inlineStr"/>
       <c r="AT134" t="inlineStr"/>
+      <c r="AU134" t="inlineStr"/>
+      <c r="AV134" t="inlineStr"/>
+      <c r="AW134" t="inlineStr"/>
+      <c r="AX134" t="inlineStr"/>
+      <c r="AY134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -18319,6 +19037,11 @@
       <c r="AR135" t="inlineStr"/>
       <c r="AS135" t="inlineStr"/>
       <c r="AT135" t="inlineStr"/>
+      <c r="AU135" t="inlineStr"/>
+      <c r="AV135" t="inlineStr"/>
+      <c r="AW135" t="inlineStr"/>
+      <c r="AX135" t="inlineStr"/>
+      <c r="AY135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -18451,6 +19174,11 @@
       <c r="AR136" t="inlineStr"/>
       <c r="AS136" t="inlineStr"/>
       <c r="AT136" t="inlineStr"/>
+      <c r="AU136" t="inlineStr"/>
+      <c r="AV136" t="inlineStr"/>
+      <c r="AW136" t="inlineStr"/>
+      <c r="AX136" t="inlineStr"/>
+      <c r="AY136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -18583,6 +19311,11 @@
       <c r="AR137" t="inlineStr"/>
       <c r="AS137" t="inlineStr"/>
       <c r="AT137" t="inlineStr"/>
+      <c r="AU137" t="inlineStr"/>
+      <c r="AV137" t="inlineStr"/>
+      <c r="AW137" t="inlineStr"/>
+      <c r="AX137" t="inlineStr"/>
+      <c r="AY137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -18715,6 +19448,11 @@
       <c r="AR138" t="inlineStr"/>
       <c r="AS138" t="inlineStr"/>
       <c r="AT138" t="inlineStr"/>
+      <c r="AU138" t="inlineStr"/>
+      <c r="AV138" t="inlineStr"/>
+      <c r="AW138" t="inlineStr"/>
+      <c r="AX138" t="inlineStr"/>
+      <c r="AY138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -18847,6 +19585,11 @@
       <c r="AR139" t="inlineStr"/>
       <c r="AS139" t="inlineStr"/>
       <c r="AT139" t="inlineStr"/>
+      <c r="AU139" t="inlineStr"/>
+      <c r="AV139" t="inlineStr"/>
+      <c r="AW139" t="inlineStr"/>
+      <c r="AX139" t="inlineStr"/>
+      <c r="AY139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -18979,6 +19722,11 @@
       <c r="AR140" t="inlineStr"/>
       <c r="AS140" t="inlineStr"/>
       <c r="AT140" t="inlineStr"/>
+      <c r="AU140" t="inlineStr"/>
+      <c r="AV140" t="inlineStr"/>
+      <c r="AW140" t="inlineStr"/>
+      <c r="AX140" t="inlineStr"/>
+      <c r="AY140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -19111,6 +19859,11 @@
       <c r="AR141" t="inlineStr"/>
       <c r="AS141" t="inlineStr"/>
       <c r="AT141" t="inlineStr"/>
+      <c r="AU141" t="inlineStr"/>
+      <c r="AV141" t="inlineStr"/>
+      <c r="AW141" t="inlineStr"/>
+      <c r="AX141" t="inlineStr"/>
+      <c r="AY141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -19243,6 +19996,11 @@
       <c r="AR142" t="inlineStr"/>
       <c r="AS142" t="inlineStr"/>
       <c r="AT142" t="inlineStr"/>
+      <c r="AU142" t="inlineStr"/>
+      <c r="AV142" t="inlineStr"/>
+      <c r="AW142" t="inlineStr"/>
+      <c r="AX142" t="inlineStr"/>
+      <c r="AY142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -19375,6 +20133,11 @@
       <c r="AR143" t="inlineStr"/>
       <c r="AS143" t="inlineStr"/>
       <c r="AT143" t="inlineStr"/>
+      <c r="AU143" t="inlineStr"/>
+      <c r="AV143" t="inlineStr"/>
+      <c r="AW143" t="inlineStr"/>
+      <c r="AX143" t="inlineStr"/>
+      <c r="AY143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -19507,6 +20270,11 @@
       <c r="AR144" t="inlineStr"/>
       <c r="AS144" t="inlineStr"/>
       <c r="AT144" t="inlineStr"/>
+      <c r="AU144" t="inlineStr"/>
+      <c r="AV144" t="inlineStr"/>
+      <c r="AW144" t="inlineStr"/>
+      <c r="AX144" t="inlineStr"/>
+      <c r="AY144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -19639,6 +20407,11 @@
       <c r="AR145" t="inlineStr"/>
       <c r="AS145" t="inlineStr"/>
       <c r="AT145" t="inlineStr"/>
+      <c r="AU145" t="inlineStr"/>
+      <c r="AV145" t="inlineStr"/>
+      <c r="AW145" t="inlineStr"/>
+      <c r="AX145" t="inlineStr"/>
+      <c r="AY145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -19771,6 +20544,11 @@
       <c r="AR146" t="inlineStr"/>
       <c r="AS146" t="inlineStr"/>
       <c r="AT146" t="inlineStr"/>
+      <c r="AU146" t="inlineStr"/>
+      <c r="AV146" t="inlineStr"/>
+      <c r="AW146" t="inlineStr"/>
+      <c r="AX146" t="inlineStr"/>
+      <c r="AY146" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>